<commit_message>
TFR changes and scaling
</commit_message>
<xml_diff>
--- a/TFR_Lat_Lon.xlsx
+++ b/TFR_Lat_Lon.xlsx
@@ -1,41 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Karrnidh Arora\Desktop\internships\MDP Project\update\integration\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07690DB6-F691-48D4-9094-F4C16B5028CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
-    <t>Vertex</t>
-  </si>
-  <si>
     <t>Lat_dd</t>
   </si>
   <si>
     <t>Lon_dd</t>
   </si>
+  <si>
+    <t>Vertex</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -72,21 +66,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -124,7 +110,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -158,7 +144,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -193,10 +178,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -369,22 +353,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -392,161 +376,95 @@
         <v>26.5</v>
       </c>
       <c r="C2">
-        <v>-97.2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+        <v>-83.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>26.8</v>
+        <v>26.5</v>
       </c>
       <c r="C3">
-        <v>-96.5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+        <v>-79.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4">
-        <v>27.2</v>
+        <v>25.5</v>
       </c>
       <c r="C4">
-        <v>-95</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+        <v>-78.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C5">
-        <v>-93</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+        <v>-78</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6">
-        <v>26.5</v>
+        <v>22.5</v>
       </c>
       <c r="C6">
-        <v>-91</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+        <v>-79.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7">
-        <v>25.8</v>
+        <v>22.5</v>
       </c>
       <c r="C7">
-        <v>-89.5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+        <v>-82.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8">
-        <v>25</v>
+        <v>23.5</v>
       </c>
       <c r="C8">
-        <v>-88</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+        <v>-84</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C9">
-        <v>-87.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+        <v>-84</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10">
-        <v>23.5</v>
+        <v>26.5</v>
       </c>
       <c r="C10">
-        <v>-89</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11">
-        <v>23</v>
-      </c>
-      <c r="C11">
-        <v>-91</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12">
-        <v>23.2</v>
-      </c>
-      <c r="C12">
-        <v>-93.5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13">
-        <v>23.8</v>
-      </c>
-      <c r="C13">
-        <v>-95.5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14">
-        <v>24.5</v>
-      </c>
-      <c r="C14">
-        <v>-96.8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15">
-        <v>25.5</v>
-      </c>
-      <c r="C15">
-        <v>-97.3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16">
-        <v>26.5</v>
-      </c>
-      <c r="C16">
-        <v>-97.2</v>
+        <v>-83.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>